<commit_message>
Refactor authentication and handler documentation; remove unused LLM worker handler
</commit_message>
<xml_diff>
--- a/docs/banco-di-prova-modelli.xlsx
+++ b/docs/banco-di-prova-modelli.xlsx
@@ -198,6 +198,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>banco di prova</author>
+  </authors>
+  <commentList>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Scrivi qui il tuo nome per dividervi le 10 righe in due, oppure lascialo vuoto se le fate entrambi (vedi Leggimi, sezione 1bis).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -489,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -565,46 +580,174 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>1bis. Come scattare e mandare le 10 foto della scheda 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Basta il telefono: un capo per foto, ben visibile, senza altri capi intorno. Va bene la luce di casa reale, anche imperfetta — anzi è voluto (vedi cosa deve coprire ogni foto nella colonna «caratteristica» della scheda 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Salva ogni foto in JPEG, indicativamente sotto i 300 KB: non serve più risoluzione di quella che userebbe davvero l'app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Per il campione con l'etichetta (l'ultima riga, c10), assicurati che il testo del cartellino sia leggibile nella foto, non solo presente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Siete in due: scrivi il tuo nome nella colonna «chi fotografa» della scheda 1 per dividervi le 10 righe, oppure fatele entrambi (10 a testa, 20 foto totali) per un confronto più solido — vanno bene entrambe le strade, basta che vi accordiate lì.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Quando mandi le foto, chiamale con il tuo nome davanti al nome già previsto in «foto (non modificare)», es. marouan_c01.jpg — così si capisce subito di chi è ognuna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>2. Giudizio soggettivo sull'app</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Ogni volta che provate la chat di Tela con foto vere, aggiungete una riga: cosa avete chiesto, che provider era attivo, se la risposta vi è sembrata naturale e l'outfit proposto sensato. Non serve saper programmare: è solo la vostra impressione.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2bis. Le domande da fare alla chat (per la scheda 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Usa sempre le stesse domande per ogni modello che provi, così il confronto è equo. Una riga per domanda nella scheda «Giudizio soggettivo», ripeti il blocco di domande per ogni modello:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>1. Un'occasione concreta: «Cosa mi metto oggi per un colloquio / una cena / la palestra?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2. Una richiesta vaga, senza dettagli: «Vestimi bene per stasera» — guarda se fa domande o inventa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>3. Qualcosa che il tuo armadio caricato non può soddisfare davvero (es. chiedi un outfit invernale se hai caricato solo capi estivi) — controlla se INVENTA un capo che non hai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>4. Una domanda su un capo preciso che hai caricato: «Come abbino [questo capo]?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>5. Un seguito nella stessa conversazione (es. «e se piove?») — verifica se si ricorda il contesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>6. Una domanda su un capo che sai per certo di NON aver caricato — deve ammettere di non saperlo, non inventarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Nella colonna «ha inventato o sbagliato qualcosa?» scrivi sempre una nota concreta quando succede (es. «ha detto che ho una giacca blu, non ce l'ho»): è il segnale più importante di tutto il foglio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>3. Voti immagini generate</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Per ogni immagine che Tela genera pulendo la foto di un capo, un voto da 1 a 5 su tre cose: il colore è rimasto fedele? Lo sfondo è pulito? Ci sono artefatti strani (dita in più, tessuto deformato)? L'immagine la trovate dove chi ha lanciato il test ve l'ha condivisa.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Alla fine, confrontate le tre schede e decidete insieme quale provider/modello usare — il costo e la velocità li trovate nella schermata «Valutazione modelli» dentro l'app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>4. Come mandarmi tutto quando avete finito</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="38" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Mandate questo file Excel compilato più le foto (via file diretti, email, drive — quello che vi è più comodo): niente da installare, nessun altro passaggio da fare voi.</t>
         </is>
       </c>
     </row>
@@ -619,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -634,6 +777,7 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -695,6 +839,11 @@
       <c r="L1" s="5" t="inlineStr">
         <is>
           <t>lavaggio</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>chi fotografa</t>
         </is>
       </c>
     </row>
@@ -723,6 +872,7 @@
       <c r="J2" s="7" t="n"/>
       <c r="K2" s="7" t="n"/>
       <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -749,6 +899,7 @@
       <c r="J3" s="7" t="n"/>
       <c r="K3" s="7" t="n"/>
       <c r="L3" s="7" t="n"/>
+      <c r="M3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -775,6 +926,7 @@
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -801,6 +953,7 @@
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
       <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -827,6 +980,7 @@
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -853,6 +1007,7 @@
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
       <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -879,6 +1034,7 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -905,6 +1061,7 @@
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
       <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -931,6 +1088,7 @@
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -957,6 +1115,7 @@
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -966,6 +1125,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>